<commit_message>
Order McNemar Table3 rows by QID
</commit_message>
<xml_diff>
--- a/mcnemar/Table3_formatted.xlsx
+++ b/mcnemar/Table3_formatted.xlsx
@@ -1871,161 +1871,161 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>68.7</t>
+          <t>88.0</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>86.0**</t>
+          <t>90.7</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>71.3</t>
+          <t>91.3</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>70.1</t>
+          <t>73.8</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>82.1</t>
+          <t>88.5*</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>61.2</t>
+          <t>86.9</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>62.7</t>
+          <t>87.3</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>80.7**</t>
+          <t>90.7</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>88.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>43.9</t>
+          <t>76.7</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>68.4**</t>
+          <t>91.8*</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>29.8</t>
+          <t>83.6</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>88.0</t>
+          <t>68.7</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>90.7</t>
+          <t>86.0**</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>91.3</t>
+          <t>71.3</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>73.8</t>
+          <t>70.1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>88.5*</t>
+          <t>82.1</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>86.9</t>
+          <t>61.2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>87.3</t>
+          <t>62.7</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>90.7</t>
+          <t>80.7**</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>88.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>76.7</t>
+          <t>43.9</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>91.8*</t>
+          <t>68.4**</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>83.6</t>
+          <t>29.8</t>
         </is>
       </c>
     </row>
@@ -2118,241 +2118,241 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>From what years were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>51.3</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>72.7**</t>
+          <t>86.0</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>78.0**</t>
+          <t>92.7*</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>85.1</t>
+          <t>82.4</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>55.2</t>
+          <t>80.0</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>70.1</t>
+          <t>92.9*</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>43.3</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>70.7**</t>
+          <t>70.7</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>72.0**</t>
+          <t>75.3</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>66.7</t>
+          <t>62.4</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>40.4</t>
+          <t>65.6</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>49.1</t>
+          <t>73.6*</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>From what years were the sequenced samples obtained?</t>
+          <t>What method was used for sequencing?</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>84.0</t>
+          <t>78.7</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>86.0</t>
+          <t>85.3</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>92.7*</t>
+          <t>87.3</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>82.4</t>
+          <t>61.7</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>75.3</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>92.9*</t>
+          <t>80.2*</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>66.7</t>
+          <t>83.3</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>70.7</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>75.3</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>62.4</t>
+          <t>68.9</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>65.6</t>
+          <t>62.3</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>73.6*</t>
+          <t>85.2*</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>What method was used for sequencing?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>78.7</t>
+          <t>51.3</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>85.3</t>
+          <t>72.7**</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>87.3</t>
+          <t>78.0**</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>61.7</t>
+          <t>85.1</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>75.3</t>
+          <t>55.2</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>80.2*</t>
+          <t>70.1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>83.3</t>
+          <t>43.3</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>84.0</t>
+          <t>70.7**</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>72.0**</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>68.9</t>
+          <t>66.7</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>62.3</t>
+          <t>40.4</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>85.2*</t>
+          <t>49.1</t>
         </is>
       </c>
     </row>
@@ -2405,241 +2405,241 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>69.3</t>
+          <t>73.3</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>74.7</t>
+          <t>73.3</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>78.0</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>48.9</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>62.2</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>81.1**</t>
+          <t>81.0*</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>From what years were the sequenced samples obtained?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>80.7</t>
+          <t>69.3</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>77.3</t>
+          <t>74.7</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>84.0</t>
+          <t>80.0</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>71.8</t>
+          <t>48.9</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>62.4</t>
+          <t>62.2</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>97.6**</t>
+          <t>81.1**</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>From what years were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>80.7</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>55.3</t>
+          <t>77.3</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>78.7**</t>
+          <t>84.0</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>53.6</t>
+          <t>71.8</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>47.2</t>
+          <t>62.4</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>79.2**</t>
+          <t>97.6**</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>81.3</t>
+          <t>55.3</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>78.7**</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>53.6</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>47.2</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>91.8**</t>
+          <t>79.2**</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>76.0</t>
+          <t>79.3</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>79.3</t>
+          <t>81.3</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>73.3</t>
+          <t>80.0</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>74.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>65.8</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>97.3**</t>
+          <t>91.8**</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>76.0</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>79.3</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
           <t>73.3</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>73.3</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>78.0</t>
-        </is>
-      </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>64.0</t>
+          <t>74.0</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>65.8</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>81.0*</t>
+          <t>97.3**</t>
         </is>
       </c>
     </row>

</xml_diff>